<commit_message>
Add audio/images assets and update content pipeline
- Add slide-1.png and slide_1.mp3 to frontend/public
- Update update-content.sh to auto-sync images and audios
- Update content.json and Excel source
</commit_message>
<xml_diff>
--- a/learnflow-content.xlsx
+++ b/learnflow-content.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vuanhtuan/Desktop/DONG A/WEB/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vuanhtuan/Desktop/DONG A/learnflow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E87E522F-9F2C-444E-9410-82634D72246F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{54F6FA40-72C8-DD41-B9DD-60AFDEFD21F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20460" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -137,12 +137,6 @@
     <t>image+audio</t>
   </si>
   <si>
-    <t>python-intro.jpg</t>
-  </si>
-  <si>
-    <t>python-intro.mp3</t>
-  </si>
-  <si>
     <t>Giới thiệu Python · 1:42</t>
   </si>
   <si>
@@ -348,6 +342,12 @@
   </si>
   <si>
     <t>Khởi tạo dự án</t>
+  </si>
+  <si>
+    <t>slide-1.png</t>
+  </si>
+  <si>
+    <t>slide_1.mp3</t>
   </si>
 </sst>
 </file>
@@ -1047,13 +1047,13 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>8</v>
@@ -1064,13 +1064,13 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>88</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>90</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>7</v>
@@ -1137,13 +1137,13 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D3" s="4">
         <v>1</v>
@@ -1152,13 +1152,13 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D4" s="6">
         <v>2</v>
@@ -1167,13 +1167,13 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D5" s="8">
         <v>3</v>
@@ -1250,13 +1250,13 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>19</v>
@@ -1271,13 +1271,13 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>21</v>
@@ -1292,13 +1292,13 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>22</v>
@@ -1313,13 +1313,13 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>22</v>
@@ -1334,13 +1334,13 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>22</v>
@@ -1434,7 +1434,7 @@
     </row>
     <row r="3" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B3" s="14">
         <v>1</v>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="4" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B4" s="18">
         <v>2</v>
@@ -1462,44 +1462,44 @@
         <v>36</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>37</v>
+        <v>105</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>38</v>
+        <v>106</v>
       </c>
       <c r="F4" s="18">
         <v>102</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H4" s="17"/>
       <c r="I4" s="17"/>
     </row>
     <row r="5" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B5" s="22">
         <v>3</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E5" s="21"/>
       <c r="F5" s="22"/>
       <c r="G5" s="21"/>
       <c r="H5" s="21" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="I5" s="21"/>
     </row>
     <row r="6" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B6" s="14">
         <v>1</v>
@@ -1508,7 +1508,7 @@
         <v>34</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E6" s="13"/>
       <c r="F6" s="14"/>
@@ -1518,16 +1518,16 @@
     </row>
     <row r="7" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B7" s="26">
         <v>2</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E7" s="25"/>
       <c r="F7" s="26"/>
@@ -1539,28 +1539,28 @@
     </row>
     <row r="8" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B8" s="22">
         <v>3</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D8" s="24" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E8" s="21"/>
       <c r="F8" s="22"/>
       <c r="G8" s="21"/>
       <c r="H8" s="21" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="I8" s="21"/>
     </row>
     <row r="9" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B9" s="14">
         <v>1</v>
@@ -1569,7 +1569,7 @@
         <v>34</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E9" s="13"/>
       <c r="F9" s="14"/>
@@ -1579,7 +1579,7 @@
     </row>
     <row r="10" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B10" s="18">
         <v>2</v>
@@ -1588,16 +1588,16 @@
         <v>36</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F10" s="18">
         <v>125</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="H10" s="17"/>
       <c r="I10" s="17" t="s">
@@ -1606,16 +1606,16 @@
     </row>
     <row r="11" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B11" s="26">
         <v>3</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E11" s="25"/>
       <c r="F11" s="26"/>
@@ -1627,16 +1627,16 @@
     </row>
     <row r="12" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B12" s="30">
         <v>4</v>
       </c>
       <c r="C12" s="31" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D12" s="32" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E12" s="29"/>
       <c r="F12" s="30"/>
@@ -1646,7 +1646,7 @@
     </row>
     <row r="14" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="36" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B14" s="34"/>
       <c r="C14" s="34"/>
@@ -1659,7 +1659,7 @@
     </row>
     <row r="15" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="33" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B15" s="34"/>
       <c r="C15" s="34"/>
@@ -1672,7 +1672,7 @@
     </row>
     <row r="16" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="33" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B16" s="34"/>
       <c r="C16" s="34"/>
@@ -1705,7 +1705,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="40" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B1" s="34"/>
       <c r="C1" s="34"/>
@@ -1715,7 +1715,7 @@
     </row>
     <row r="3" spans="1:6" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="38" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B3" s="34"/>
       <c r="C3" s="34"/>
@@ -1725,7 +1725,7 @@
     </row>
     <row r="4" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="37" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B4" s="34"/>
       <c r="C4" s="34"/>
@@ -1735,7 +1735,7 @@
     </row>
     <row r="5" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="37" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B5" s="34"/>
       <c r="C5" s="34"/>
@@ -1745,7 +1745,7 @@
     </row>
     <row r="6" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="37" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B6" s="34"/>
       <c r="C6" s="34"/>
@@ -1755,7 +1755,7 @@
     </row>
     <row r="7" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="37" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B7" s="34"/>
       <c r="C7" s="34"/>
@@ -1765,7 +1765,7 @@
     </row>
     <row r="8" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="39" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B8" s="34"/>
       <c r="C8" s="34"/>
@@ -1775,7 +1775,7 @@
     </row>
     <row r="10" spans="1:6" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="38" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B10" s="34"/>
       <c r="C10" s="34"/>
@@ -1785,7 +1785,7 @@
     </row>
     <row r="11" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="37" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B11" s="34"/>
       <c r="C11" s="34"/>
@@ -1795,7 +1795,7 @@
     </row>
     <row r="12" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="37" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B12" s="34"/>
       <c r="C12" s="34"/>
@@ -1805,7 +1805,7 @@
     </row>
     <row r="13" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="37" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B13" s="34"/>
       <c r="C13" s="34"/>
@@ -1815,7 +1815,7 @@
     </row>
     <row r="14" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="37" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B14" s="34"/>
       <c r="C14" s="34"/>
@@ -1825,7 +1825,7 @@
     </row>
     <row r="15" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="37" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B15" s="34"/>
       <c r="C15" s="34"/>
@@ -1835,7 +1835,7 @@
     </row>
     <row r="16" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="37" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B16" s="34"/>
       <c r="C16" s="34"/>
@@ -1845,7 +1845,7 @@
     </row>
     <row r="17" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="37" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B17" s="34"/>
       <c r="C17" s="34"/>
@@ -1855,7 +1855,7 @@
     </row>
     <row r="19" spans="1:6" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="38" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B19" s="34"/>
       <c r="C19" s="34"/>
@@ -1865,7 +1865,7 @@
     </row>
     <row r="20" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="37" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B20" s="34"/>
       <c r="C20" s="34"/>
@@ -1875,7 +1875,7 @@
     </row>
     <row r="22" spans="1:6" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="38" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B22" s="34"/>
       <c r="C22" s="34"/>
@@ -1885,7 +1885,7 @@
     </row>
     <row r="23" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="37" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B23" s="34"/>
       <c r="C23" s="34"/>
@@ -1895,7 +1895,7 @@
     </row>
     <row r="24" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="37" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B24" s="34"/>
       <c r="C24" s="34"/>
@@ -1905,7 +1905,7 @@
     </row>
     <row r="25" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="37" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B25" s="34"/>
       <c r="C25" s="34"/>
@@ -1915,7 +1915,7 @@
     </row>
     <row r="26" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="37" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B26" s="34"/>
       <c r="C26" s="34"/>
@@ -1925,7 +1925,7 @@
     </row>
     <row r="28" spans="1:6" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="38" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B28" s="34"/>
       <c r="C28" s="34"/>
@@ -1935,7 +1935,7 @@
     </row>
     <row r="29" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="37" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B29" s="34"/>
       <c r="C29" s="34"/>
@@ -1945,7 +1945,7 @@
     </row>
     <row r="30" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="39" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B30" s="34"/>
       <c r="C30" s="34"/>
@@ -1955,7 +1955,7 @@
     </row>
     <row r="31" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="37" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B31" s="34"/>
       <c r="C31" s="34"/>
@@ -1965,7 +1965,7 @@
     </row>
     <row r="32" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="37" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B32" s="34"/>
       <c r="C32" s="34"/>

</xml_diff>